<commit_message>
R1. Impossible to replicate. Missing datasets. README lacking crucial information
</commit_message>
<xml_diff>
--- a/package-output-map.xlsx
+++ b/package-output-map.xlsx
@@ -1,31 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/floswald/git/JPEtemplate/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elian\Desktop\MS20241468_Deposit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{067DD2C7-24FE-2447-A5A8-8F6542C7C06E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D196D3A-5709-465C-914E-412B73BA9F8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="21900" windowHeight="12060" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
-  <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="60">
   <si>
     <t>Data Preparation Program</t>
   </si>
@@ -46,6 +41,165 @@
   </si>
   <si>
     <t>In-text numbers</t>
+  </si>
+  <si>
+    <t>Figure 1</t>
+  </si>
+  <si>
+    <t>2b_figures_descriptives.do</t>
+  </si>
+  <si>
+    <t>p.3 &amp; 39: "in the absence of immigration, union density 1900-1920 would have been ~22% lower" (also ~31% for skilled)</t>
+  </si>
+  <si>
+    <t>2c_results_main.do</t>
+  </si>
+  <si>
+    <t>195–197</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Figure 2</t>
+  </si>
+  <si>
+    <t>2a_sumstats.do</t>
+  </si>
+  <si>
+    <t>Figure 3</t>
+  </si>
+  <si>
+    <t>2e_results_robustness.do</t>
+  </si>
+  <si>
+    <t>Figure 4</t>
+  </si>
+  <si>
+    <t>Figure 5</t>
+  </si>
+  <si>
+    <t>Table 1</t>
+  </si>
+  <si>
+    <t>Table 2</t>
+  </si>
+  <si>
+    <t>Table 3</t>
+  </si>
+  <si>
+    <t>Table 4</t>
+  </si>
+  <si>
+    <t>Table 5</t>
+  </si>
+  <si>
+    <t>Table 6</t>
+  </si>
+  <si>
+    <t>Table 7</t>
+  </si>
+  <si>
+    <t>Table 8</t>
+  </si>
+  <si>
+    <t>Figure A.1</t>
+  </si>
+  <si>
+    <t>Figure A.4</t>
+  </si>
+  <si>
+    <t>Figure A.5</t>
+  </si>
+  <si>
+    <t>Figure G.1</t>
+  </si>
+  <si>
+    <t>2f_rotemberg_weights.do</t>
+  </si>
+  <si>
+    <t>Figure H.1</t>
+  </si>
+  <si>
+    <t>Table A.2</t>
+  </si>
+  <si>
+    <t>Table A.3</t>
+  </si>
+  <si>
+    <t>Table A.4</t>
+  </si>
+  <si>
+    <t>2d_results_extra.do</t>
+  </si>
+  <si>
+    <t>Table A.5</t>
+  </si>
+  <si>
+    <t>Table A.6</t>
+  </si>
+  <si>
+    <t>Table A.7</t>
+  </si>
+  <si>
+    <t>Table A.8</t>
+  </si>
+  <si>
+    <t>Table A.9</t>
+  </si>
+  <si>
+    <t>Table A.10</t>
+  </si>
+  <si>
+    <t>Table A.11</t>
+  </si>
+  <si>
+    <t>Table B.2</t>
+  </si>
+  <si>
+    <t>Table G.1</t>
+  </si>
+  <si>
+    <t>Table G.2</t>
+  </si>
+  <si>
+    <t>Figure B.2</t>
+  </si>
+  <si>
+    <t>Figure B.1</t>
+  </si>
+  <si>
+    <t>1e_weather_shocks.do</t>
+  </si>
+  <si>
+    <t>Table B.1</t>
+  </si>
+  <si>
+    <t>Table A.1</t>
+  </si>
+  <si>
+    <t>Figure A.2</t>
+  </si>
+  <si>
+    <t>Figure A.3</t>
+  </si>
+  <si>
+    <t>Table E.1</t>
+  </si>
+  <si>
+    <t>Table F.1</t>
+  </si>
+  <si>
+    <t>?</t>
+  </si>
+  <si>
+    <t>/</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>no</t>
   </si>
 </sst>
 </file>
@@ -434,22 +588,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D18"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:L40"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.5" customWidth="1"/>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26" customWidth="1"/>
+    <col min="2" max="2" width="17" customWidth="1"/>
     <col min="3" max="3" width="13" customWidth="1"/>
-    <col min="5" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="2" customWidth="1"/>
+    <col min="5" max="5" width="26" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="28" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.88671875" customWidth="1"/>
+    <col min="9" max="9" width="65" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -459,49 +614,569 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="E2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2">
+        <v>66</v>
+      </c>
+      <c r="H2" t="s">
+        <v>58</v>
+      </c>
+      <c r="I2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K2" t="s">
+        <v>11</v>
+      </c>
+      <c r="L2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3">
+        <v>50</v>
+      </c>
+      <c r="H3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="E4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4">
+        <v>1536</v>
+      </c>
+      <c r="H4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="E5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5">
+        <v>229</v>
+      </c>
+      <c r="H5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="E6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6">
+        <v>427</v>
+      </c>
+      <c r="H6" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="E7" t="s">
+        <v>19</v>
+      </c>
+      <c r="F7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7">
+        <v>155</v>
+      </c>
+      <c r="H7" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B8" s="3"/>
+      <c r="E8" t="s">
+        <v>20</v>
+      </c>
+      <c r="F8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G8">
+        <v>42</v>
+      </c>
+      <c r="H8" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B9" s="3"/>
+      <c r="E9" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" t="s">
+        <v>10</v>
+      </c>
+      <c r="G9">
+        <v>80</v>
+      </c>
+      <c r="H9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A10" s="3"/>
+      <c r="B10" s="3"/>
+      <c r="E10" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10" t="s">
+        <v>10</v>
+      </c>
+      <c r="G10">
+        <v>205</v>
+      </c>
+      <c r="H10" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A11" s="3"/>
+      <c r="B11" s="3"/>
+      <c r="E11" t="s">
+        <v>23</v>
+      </c>
+      <c r="F11" t="s">
+        <v>10</v>
+      </c>
+      <c r="G11">
+        <v>289</v>
+      </c>
+      <c r="H11" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="E12" t="s">
+        <v>24</v>
+      </c>
+      <c r="F12" t="s">
+        <v>10</v>
+      </c>
+      <c r="G12">
+        <v>342</v>
+      </c>
+      <c r="H12" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="E13" t="s">
+        <v>25</v>
+      </c>
+      <c r="F13" t="s">
+        <v>10</v>
+      </c>
+      <c r="G13">
+        <v>484</v>
+      </c>
+      <c r="H13" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="E14" t="s">
+        <v>26</v>
+      </c>
+      <c r="F14" t="s">
+        <v>10</v>
+      </c>
+      <c r="G14">
+        <v>560</v>
+      </c>
+      <c r="H14" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="E15" t="s">
+        <v>27</v>
+      </c>
+      <c r="F15" t="s">
+        <v>8</v>
+      </c>
+      <c r="G15">
+        <v>40</v>
+      </c>
+      <c r="H15" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="E16" t="s">
+        <v>28</v>
+      </c>
+      <c r="F16" t="s">
+        <v>14</v>
+      </c>
+      <c r="G16">
+        <v>285</v>
+      </c>
+      <c r="H16" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="17" spans="5:8" x14ac:dyDescent="0.3">
+      <c r="E17" t="s">
+        <v>29</v>
+      </c>
+      <c r="F17" t="s">
+        <v>10</v>
+      </c>
+      <c r="G17">
+        <v>808</v>
+      </c>
+      <c r="H17" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="18" spans="5:8" x14ac:dyDescent="0.3">
+      <c r="E18" t="s">
+        <v>30</v>
+      </c>
+      <c r="F18" t="s">
+        <v>31</v>
+      </c>
+      <c r="G18">
+        <v>254</v>
+      </c>
+      <c r="H18" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="19" spans="5:8" x14ac:dyDescent="0.3">
+      <c r="E19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F19" t="s">
+        <v>14</v>
+      </c>
+      <c r="G19">
+        <v>355</v>
+      </c>
+      <c r="H19" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="20" spans="5:8" x14ac:dyDescent="0.3">
+      <c r="E20" t="s">
+        <v>33</v>
+      </c>
+      <c r="F20" t="s">
+        <v>14</v>
+      </c>
+      <c r="G20">
+        <v>199</v>
+      </c>
+      <c r="H20" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="21" spans="5:8" x14ac:dyDescent="0.3">
+      <c r="E21" t="s">
+        <v>34</v>
+      </c>
+      <c r="F21" t="s">
+        <v>14</v>
+      </c>
+      <c r="G21">
+        <v>236</v>
+      </c>
+      <c r="H21" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="22" spans="5:8" x14ac:dyDescent="0.3">
+      <c r="E22" t="s">
+        <v>35</v>
+      </c>
+      <c r="F22" t="s">
+        <v>36</v>
+      </c>
+      <c r="G22">
+        <v>38</v>
+      </c>
+      <c r="H22" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="23" spans="5:8" x14ac:dyDescent="0.3">
+      <c r="E23" t="s">
+        <v>37</v>
+      </c>
+      <c r="F23" t="s">
+        <v>10</v>
+      </c>
+      <c r="G23">
+        <v>409</v>
+      </c>
+      <c r="H23" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="24" spans="5:8" x14ac:dyDescent="0.3">
+      <c r="E24" t="s">
+        <v>38</v>
+      </c>
+      <c r="F24" t="s">
+        <v>10</v>
+      </c>
+      <c r="G24">
+        <v>759</v>
+      </c>
+      <c r="H24" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="25" spans="5:8" x14ac:dyDescent="0.3">
+      <c r="E25" t="s">
+        <v>39</v>
+      </c>
+      <c r="F25" t="s">
+        <v>10</v>
+      </c>
+      <c r="G25">
+        <v>858</v>
+      </c>
+      <c r="H25" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="26" spans="5:8" x14ac:dyDescent="0.3">
+      <c r="E26" t="s">
+        <v>40</v>
+      </c>
+      <c r="F26" t="s">
+        <v>36</v>
+      </c>
+      <c r="G26">
+        <v>94</v>
+      </c>
+      <c r="H26" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="27" spans="5:8" x14ac:dyDescent="0.3">
+      <c r="E27" t="s">
+        <v>41</v>
+      </c>
+      <c r="F27" t="s">
+        <v>36</v>
+      </c>
+      <c r="G27">
+        <v>149</v>
+      </c>
+      <c r="H27" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="28" spans="5:8" x14ac:dyDescent="0.3">
+      <c r="E28" t="s">
+        <v>42</v>
+      </c>
+      <c r="F28" t="s">
+        <v>36</v>
+      </c>
+      <c r="G28">
+        <v>210</v>
+      </c>
+      <c r="H28" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="29" spans="5:8" x14ac:dyDescent="0.3">
+      <c r="E29" t="s">
+        <v>43</v>
+      </c>
+      <c r="F29" t="s">
+        <v>36</v>
+      </c>
+      <c r="G29">
+        <v>278</v>
+      </c>
+      <c r="H29" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="30" spans="5:8" x14ac:dyDescent="0.3">
+      <c r="E30" t="s">
+        <v>44</v>
+      </c>
+      <c r="F30" t="s">
+        <v>16</v>
+      </c>
+      <c r="G30">
+        <v>44</v>
+      </c>
+      <c r="H30" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="31" spans="5:8" x14ac:dyDescent="0.3">
+      <c r="E31" t="s">
+        <v>45</v>
+      </c>
+      <c r="F31" t="s">
+        <v>31</v>
+      </c>
+      <c r="G31">
+        <v>196</v>
+      </c>
+      <c r="H31" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="32" spans="5:8" x14ac:dyDescent="0.3">
+      <c r="E32" t="s">
+        <v>46</v>
+      </c>
+      <c r="F32" t="s">
+        <v>16</v>
+      </c>
+      <c r="G32">
+        <v>44</v>
+      </c>
+      <c r="H32" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="33" spans="5:8" x14ac:dyDescent="0.3">
+      <c r="E33" t="s">
+        <v>47</v>
+      </c>
+      <c r="F33" t="s">
+        <v>16</v>
+      </c>
+      <c r="G33">
+        <v>221</v>
+      </c>
+      <c r="H33" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="34" spans="5:8" x14ac:dyDescent="0.3">
+      <c r="E34" t="s">
+        <v>48</v>
+      </c>
+      <c r="F34" t="s">
+        <v>49</v>
+      </c>
+      <c r="G34">
+        <v>189</v>
+      </c>
+      <c r="H34" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="35" spans="5:8" x14ac:dyDescent="0.3">
+      <c r="E35" t="s">
+        <v>50</v>
+      </c>
+      <c r="F35" t="s">
+        <v>16</v>
+      </c>
+      <c r="G35">
+        <v>1137</v>
+      </c>
+      <c r="H35" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="36" spans="5:8" x14ac:dyDescent="0.3">
+      <c r="E36" t="s">
+        <v>51</v>
+      </c>
+      <c r="F36" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="37" spans="5:8" x14ac:dyDescent="0.3">
+      <c r="E37" t="s">
+        <v>52</v>
+      </c>
+      <c r="F37" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="38" spans="5:8" x14ac:dyDescent="0.3">
+      <c r="E38" t="s">
+        <v>53</v>
+      </c>
+      <c r="F38" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="39" spans="5:8" x14ac:dyDescent="0.3">
+      <c r="E39" t="s">
+        <v>54</v>
+      </c>
+      <c r="F39" t="s">
+        <v>56</v>
+      </c>
+      <c r="H39" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="40" spans="5:8" x14ac:dyDescent="0.3">
+      <c r="E40" t="s">
+        <v>55</v>
+      </c>
+      <c r="F40" t="s">
+        <v>56</v>
+      </c>
+      <c r="H40" t="s">
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>